<commit_message>
feat(template): add external template service for RFQ PDF export feat(ui): integrate PDF template editing functionality in export dialog fix(ui): simplify export button labels in ViewRequestWindow
</commit_message>
<xml_diff>
--- a/add_data/template_sqdc.xlsx
+++ b/add_data/template_sqdc.xlsx
@@ -1,45 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29429"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3DC85D3C-E813-467F-A541-C9C70AAA3AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" r:id="rId1"/>
+    <sheet name="SQDC" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
-  <si>
-    <t>Analisi SQDC - RdO N°</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+  <si>
+    <t xml:space="preserve">Analisi SQDC - RdO N°</t>
   </si>
   <si>
     <t>Data:</t>
   </si>
   <si>
-    <t>Pesi assegnati</t>
+    <t xml:space="preserve">Pesi assegnati</t>
   </si>
   <si>
     <t>%</t>
@@ -57,16 +42,16 @@
     <t>Cost:</t>
   </si>
   <si>
-    <t>aderenza del fornitore agli standard di sicurezza, alle conformità normative e al rischio finanziario e geopolitico.</t>
-  </si>
-  <si>
-    <t>capacità del fornitore di rispettare integralmente le specifiche tecniche concordate.</t>
-  </si>
-  <si>
-    <t>capacità di rispettare il tempo di consegna offerto e la flessibilità a fronte di eventuali variazioni richieste.</t>
-  </si>
-  <si>
-    <t>competitività prezzo, pagamenti e i costi accessori (es. trasporto, installazione).</t>
+    <t xml:space="preserve">aderenza del fornitore agli standard di sicurezza, alle conformità normative e al rischio finanziario e geopolitico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">capacità del fornitore di rispettare integralmente le specifiche tecniche concordate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">capacità di rispettare il tempo di consegna offerto e la flessibilità a fronte di eventuali variazioni richieste.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">competitività prezzo, pagamenti e i costi accessori (es. trasporto, installazione).</t>
   </si>
   <si>
     <t>Fornitore</t>
@@ -90,30 +75,29 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="5">
     <font>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="16"/>
+      <sz val="16.000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="10.000000"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -127,11 +111,26 @@
   </fills>
   <borders count="3">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -146,58 +145,43 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
   <cellXfs count="10">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="4" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -209,7 +193,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -255,13 +239,13 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Angsana New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -289,13 +273,13 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Cordia New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -492,134 +476,356 @@
 </a:theme>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F16"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="6" width="11.7109375" customWidth="1"/>
+    <col bestFit="1" customWidth="1" min="1" max="1" width="27.7109375"/>
+    <col customWidth="1" min="2" max="6" width="11.7109375"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="2" t="s">
+    <row r="1" ht="21">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="4" t="s">
+      <c r="B1" s="2"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="4"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="4" t="s">
+    <row r="5">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="6"/>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="4" t="s">
+      <c r="B5" s="5"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="6"/>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="4" t="s">
+      <c r="B6" s="5"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="6"/>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="4" t="s">
+      <c r="B7" s="5"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="6"/>
-    </row>
-    <row r="10" spans="1:6" ht="30" customHeight="1">
-      <c r="A10" s="7" t="s">
+      <c r="B8" s="5"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-    </row>
-    <row r="11" spans="1:6" ht="30" customHeight="1">
-      <c r="A11" s="7" t="s">
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-    </row>
-    <row r="12" spans="1:6" ht="30" customHeight="1">
-      <c r="A12" s="7" t="s">
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-    </row>
-    <row r="13" spans="1:6" ht="30" customHeight="1">
-      <c r="A13" s="7" t="s">
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="1" t="s">
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="F16" s="9" t="s">
         <v>17</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B13:F13"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
   </mergeCells>
+  <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>